<commit_message>
EDU-45: class_manager: latest progress
</commit_message>
<xml_diff>
--- a/assets/deen/madrasa/class_manager.xlsx
+++ b/assets/deen/madrasa/class_manager.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\SehhaDeveloper\src\l3\edu-journey\assets\deen\madrasa\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28E3159B-6602-4AB5-849E-6090519BBF45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F97A1FA-5CD9-41E7-B1B9-080268B6994C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="363" uniqueCount="211">
   <si>
     <t>Madrasa Class Dashboard</t>
   </si>
@@ -1022,6 +1022,15 @@
     <xf numFmtId="0" fontId="11" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1051,15 +1060,6 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2082,40 +2082,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="38.049999999999997" customHeight="1">
-      <c r="A1" s="54" t="s">
+      <c r="A1" s="57" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
-      <c r="F1" s="55"/>
-      <c r="G1" s="55"/>
-      <c r="H1" s="55"/>
-      <c r="I1" s="55"/>
-      <c r="J1" s="55"/>
-      <c r="K1" s="55"/>
-      <c r="L1" s="55"/>
-      <c r="M1" s="55"/>
-      <c r="N1" s="56"/>
+      <c r="B1" s="58"/>
+      <c r="C1" s="58"/>
+      <c r="D1" s="58"/>
+      <c r="E1" s="58"/>
+      <c r="F1" s="58"/>
+      <c r="G1" s="58"/>
+      <c r="H1" s="58"/>
+      <c r="I1" s="58"/>
+      <c r="J1" s="58"/>
+      <c r="K1" s="58"/>
+      <c r="L1" s="58"/>
+      <c r="M1" s="58"/>
+      <c r="N1" s="59"/>
     </row>
     <row r="2" spans="1:14" ht="30" customHeight="1">
-      <c r="A2" s="57" t="s">
+      <c r="A2" s="60" t="s">
         <v>197</v>
       </c>
-      <c r="B2" s="58"/>
-      <c r="C2" s="58"/>
-      <c r="D2" s="58"/>
-      <c r="E2" s="58"/>
-      <c r="F2" s="58"/>
-      <c r="G2" s="58"/>
-      <c r="H2" s="58"/>
-      <c r="I2" s="58"/>
-      <c r="J2" s="58"/>
-      <c r="K2" s="58"/>
-      <c r="L2" s="58"/>
-      <c r="M2" s="58"/>
-      <c r="N2" s="59"/>
+      <c r="B2" s="61"/>
+      <c r="C2" s="61"/>
+      <c r="D2" s="61"/>
+      <c r="E2" s="61"/>
+      <c r="F2" s="61"/>
+      <c r="G2" s="61"/>
+      <c r="H2" s="61"/>
+      <c r="I2" s="61"/>
+      <c r="J2" s="61"/>
+      <c r="K2" s="61"/>
+      <c r="L2" s="61"/>
+      <c r="M2" s="61"/>
+      <c r="N2" s="62"/>
     </row>
     <row r="3" spans="1:14" ht="25" customHeight="1">
       <c r="A3" s="2"/>
@@ -2187,11 +2187,11 @@
       </c>
       <c r="H5" s="52">
         <f>COUNTIF(AttendanceTable[Student],$B$4)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I5" s="52">
         <f>COUNTIF(ProgressTable[Student],$B$4)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J5" s="3"/>
       <c r="K5" s="3"/>
@@ -2229,14 +2229,14 @@
         <v>14</v>
       </c>
       <c r="C7" s="3"/>
-      <c r="D7" s="60" t="s">
+      <c r="D7" s="63" t="s">
         <v>198</v>
       </c>
-      <c r="E7" s="60"/>
-      <c r="F7" s="60"/>
-      <c r="G7" s="60"/>
-      <c r="H7" s="60"/>
-      <c r="I7" s="60"/>
+      <c r="E7" s="63"/>
+      <c r="F7" s="63"/>
+      <c r="G7" s="63"/>
+      <c r="H7" s="63"/>
+      <c r="I7" s="63"/>
       <c r="J7" s="3"/>
       <c r="K7" s="3"/>
       <c r="L7" s="3"/>
@@ -2297,13 +2297,13 @@
       <c r="N10" s="4"/>
     </row>
     <row r="11" spans="1:14" ht="25" customHeight="1">
-      <c r="A11" s="61" t="s">
+      <c r="A11" s="64" t="s">
         <v>199</v>
       </c>
-      <c r="B11" s="62"/>
-      <c r="C11" s="62"/>
-      <c r="D11" s="62"/>
-      <c r="E11" s="62"/>
+      <c r="B11" s="65"/>
+      <c r="C11" s="65"/>
+      <c r="D11" s="65"/>
+      <c r="E11" s="65"/>
       <c r="F11" s="3"/>
       <c r="G11" s="3"/>
       <c r="H11" s="3"/>
@@ -2519,7 +2519,7 @@
       </c>
       <c r="E20" s="3">
         <f>COUNTIFS(AttendanceTable[Student],$B$4,AttendanceTable[Status],D20)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F20" s="3"/>
       <c r="G20" s="3"/>
@@ -2731,13 +2731,13 @@
       <c r="N29" s="4"/>
     </row>
     <row r="30" spans="1:14">
-      <c r="A30" s="63" t="s">
+      <c r="A30" s="66" t="s">
         <v>204</v>
       </c>
-      <c r="B30" s="60"/>
-      <c r="C30" s="60"/>
-      <c r="D30" s="60"/>
-      <c r="E30" s="60"/>
+      <c r="B30" s="63"/>
+      <c r="C30" s="63"/>
+      <c r="D30" s="63"/>
+      <c r="E30" s="63"/>
       <c r="F30" s="3"/>
       <c r="G30" s="3"/>
       <c r="H30" s="3"/>
@@ -2749,11 +2749,11 @@
       <c r="N30" s="4"/>
     </row>
     <row r="31" spans="1:14">
-      <c r="A31" s="63"/>
-      <c r="B31" s="60"/>
-      <c r="C31" s="60"/>
-      <c r="D31" s="60"/>
-      <c r="E31" s="60"/>
+      <c r="A31" s="66"/>
+      <c r="B31" s="63"/>
+      <c r="C31" s="63"/>
+      <c r="D31" s="63"/>
+      <c r="E31" s="63"/>
       <c r="F31" s="3"/>
       <c r="G31" s="3"/>
       <c r="H31" s="3"/>
@@ -3031,30 +3031,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="38.049999999999997" customHeight="1">
-      <c r="A1" s="54" t="s">
+      <c r="A1" s="57" t="s">
         <v>184</v>
       </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
-      <c r="F1" s="55"/>
-      <c r="G1" s="55"/>
-      <c r="H1" s="55"/>
-      <c r="I1" s="56"/>
+      <c r="B1" s="58"/>
+      <c r="C1" s="58"/>
+      <c r="D1" s="58"/>
+      <c r="E1" s="58"/>
+      <c r="F1" s="58"/>
+      <c r="G1" s="58"/>
+      <c r="H1" s="58"/>
+      <c r="I1" s="59"/>
     </row>
     <row r="2" spans="1:26" ht="30" customHeight="1">
-      <c r="A2" s="57" t="s">
+      <c r="A2" s="60" t="s">
         <v>185</v>
       </c>
-      <c r="B2" s="58"/>
-      <c r="C2" s="58"/>
-      <c r="D2" s="58"/>
-      <c r="E2" s="58"/>
-      <c r="F2" s="58"/>
-      <c r="G2" s="58"/>
-      <c r="H2" s="58"/>
-      <c r="I2" s="59"/>
+      <c r="B2" s="61"/>
+      <c r="C2" s="61"/>
+      <c r="D2" s="61"/>
+      <c r="E2" s="61"/>
+      <c r="F2" s="61"/>
+      <c r="G2" s="61"/>
+      <c r="H2" s="61"/>
+      <c r="I2" s="62"/>
     </row>
     <row r="3" spans="1:26" ht="25" customHeight="1">
       <c r="A3" s="2"/>
@@ -10657,28 +10657,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="38.049999999999997" customHeight="1">
-      <c r="A1" s="54" t="s">
+      <c r="A1" s="57" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
-      <c r="F1" s="55"/>
-      <c r="G1" s="55"/>
-      <c r="H1" s="56"/>
+      <c r="B1" s="58"/>
+      <c r="C1" s="58"/>
+      <c r="D1" s="58"/>
+      <c r="E1" s="58"/>
+      <c r="F1" s="58"/>
+      <c r="G1" s="58"/>
+      <c r="H1" s="59"/>
     </row>
     <row r="2" spans="1:26" ht="30" customHeight="1">
-      <c r="A2" s="57" t="s">
+      <c r="A2" s="60" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="58"/>
-      <c r="C2" s="58"/>
-      <c r="D2" s="58"/>
-      <c r="E2" s="58"/>
-      <c r="F2" s="58"/>
-      <c r="G2" s="58"/>
-      <c r="H2" s="59"/>
+      <c r="B2" s="61"/>
+      <c r="C2" s="61"/>
+      <c r="D2" s="61"/>
+      <c r="E2" s="61"/>
+      <c r="F2" s="61"/>
+      <c r="G2" s="61"/>
+      <c r="H2" s="62"/>
     </row>
     <row r="3" spans="1:26" ht="25" customHeight="1">
       <c r="A3" s="2"/>
@@ -10880,7 +10880,9 @@
       <c r="E8" s="18">
         <v>0.47986111111111113</v>
       </c>
-      <c r="F8" s="17"/>
+      <c r="F8" s="17">
+        <v>1</v>
+      </c>
       <c r="G8" s="17"/>
       <c r="H8" s="19"/>
       <c r="I8" s="1"/>
@@ -10918,7 +10920,9 @@
       <c r="E9" s="26">
         <v>0.47986111111111113</v>
       </c>
-      <c r="F9" s="25"/>
+      <c r="F9" s="25">
+        <v>1</v>
+      </c>
       <c r="G9" s="25"/>
       <c r="H9" s="27"/>
       <c r="I9" s="1"/>
@@ -10956,7 +10960,9 @@
       <c r="E10" s="18">
         <v>0.47986111111111113</v>
       </c>
-      <c r="F10" s="17"/>
+      <c r="F10" s="17">
+        <v>1</v>
+      </c>
       <c r="G10" s="17"/>
       <c r="H10" s="19"/>
       <c r="I10" s="1"/>
@@ -10979,12 +10985,24 @@
       <c r="Z10" s="1"/>
     </row>
     <row r="11" spans="1:26" ht="25" customHeight="1">
-      <c r="A11" s="28"/>
-      <c r="B11" s="25"/>
-      <c r="C11" s="25"/>
-      <c r="D11" s="25"/>
-      <c r="E11" s="26"/>
-      <c r="F11" s="25"/>
+      <c r="A11" s="29">
+        <v>46278</v>
+      </c>
+      <c r="B11" s="25" t="s">
+        <v>38</v>
+      </c>
+      <c r="C11" s="25" t="s">
+        <v>33</v>
+      </c>
+      <c r="D11" s="25" t="s">
+        <v>34</v>
+      </c>
+      <c r="E11" s="26">
+        <v>0.52361111111111114</v>
+      </c>
+      <c r="F11" s="25">
+        <v>1</v>
+      </c>
       <c r="G11" s="25"/>
       <c r="H11" s="27"/>
       <c r="I11" s="1"/>
@@ -11007,12 +11025,24 @@
       <c r="Z11" s="1"/>
     </row>
     <row r="12" spans="1:26" ht="25" customHeight="1">
-      <c r="A12" s="29"/>
-      <c r="B12" s="17"/>
-      <c r="C12" s="17"/>
-      <c r="D12" s="17"/>
-      <c r="E12" s="18"/>
-      <c r="F12" s="17"/>
+      <c r="A12" s="29">
+        <v>46278</v>
+      </c>
+      <c r="B12" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="C12" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="D12" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="E12" s="18">
+        <v>0.52361111111111114</v>
+      </c>
+      <c r="F12" s="17">
+        <v>1</v>
+      </c>
       <c r="G12" s="17"/>
       <c r="H12" s="19"/>
       <c r="I12" s="1"/>
@@ -11035,12 +11065,24 @@
       <c r="Z12" s="1"/>
     </row>
     <row r="13" spans="1:26" ht="25" customHeight="1">
-      <c r="A13" s="28"/>
-      <c r="B13" s="25"/>
-      <c r="C13" s="25"/>
-      <c r="D13" s="25"/>
-      <c r="E13" s="26"/>
-      <c r="F13" s="25"/>
+      <c r="A13" s="29">
+        <v>46278</v>
+      </c>
+      <c r="B13" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="C13" s="25" t="s">
+        <v>33</v>
+      </c>
+      <c r="D13" s="25" t="s">
+        <v>34</v>
+      </c>
+      <c r="E13" s="26">
+        <v>0.52361111111111114</v>
+      </c>
+      <c r="F13" s="25">
+        <v>1</v>
+      </c>
       <c r="G13" s="25"/>
       <c r="H13" s="27"/>
       <c r="I13" s="1"/>
@@ -17807,24 +17849,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="38.049999999999997" customHeight="1">
-      <c r="A1" s="54" t="s">
+      <c r="A1" s="57" t="s">
         <v>40</v>
       </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
-      <c r="F1" s="56"/>
+      <c r="B1" s="58"/>
+      <c r="C1" s="58"/>
+      <c r="D1" s="58"/>
+      <c r="E1" s="58"/>
+      <c r="F1" s="59"/>
     </row>
     <row r="2" spans="1:6" ht="30" customHeight="1">
-      <c r="A2" s="57" t="s">
+      <c r="A2" s="60" t="s">
         <v>41</v>
       </c>
-      <c r="B2" s="58"/>
-      <c r="C2" s="58"/>
-      <c r="D2" s="58"/>
-      <c r="E2" s="58"/>
-      <c r="F2" s="59"/>
+      <c r="B2" s="61"/>
+      <c r="C2" s="61"/>
+      <c r="D2" s="61"/>
+      <c r="E2" s="61"/>
+      <c r="F2" s="62"/>
     </row>
     <row r="3" spans="1:6" ht="25" customHeight="1">
       <c r="A3" s="2"/>
@@ -18008,28 +18050,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="38.049999999999997" customHeight="1">
-      <c r="A1" s="54" t="s">
+      <c r="A1" s="57" t="s">
         <v>62</v>
       </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
-      <c r="F1" s="55"/>
-      <c r="G1" s="55"/>
-      <c r="H1" s="56"/>
+      <c r="B1" s="58"/>
+      <c r="C1" s="58"/>
+      <c r="D1" s="58"/>
+      <c r="E1" s="58"/>
+      <c r="F1" s="58"/>
+      <c r="G1" s="58"/>
+      <c r="H1" s="59"/>
     </row>
     <row r="2" spans="1:8" ht="30" customHeight="1">
-      <c r="A2" s="57" t="s">
+      <c r="A2" s="60" t="s">
         <v>63</v>
       </c>
-      <c r="B2" s="58"/>
-      <c r="C2" s="58"/>
-      <c r="D2" s="58"/>
-      <c r="E2" s="58"/>
-      <c r="F2" s="58"/>
-      <c r="G2" s="58"/>
-      <c r="H2" s="59"/>
+      <c r="B2" s="61"/>
+      <c r="C2" s="61"/>
+      <c r="D2" s="61"/>
+      <c r="E2" s="61"/>
+      <c r="F2" s="61"/>
+      <c r="G2" s="61"/>
+      <c r="H2" s="62"/>
     </row>
     <row r="3" spans="1:8" ht="25" customHeight="1">
       <c r="A3" s="2"/>
@@ -18209,28 +18251,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="38.049999999999997" customHeight="1">
-      <c r="A1" s="54" t="s">
+      <c r="A1" s="57" t="s">
         <v>42</v>
       </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
-      <c r="F1" s="55"/>
-      <c r="G1" s="55"/>
-      <c r="H1" s="56"/>
+      <c r="B1" s="58"/>
+      <c r="C1" s="58"/>
+      <c r="D1" s="58"/>
+      <c r="E1" s="58"/>
+      <c r="F1" s="58"/>
+      <c r="G1" s="58"/>
+      <c r="H1" s="59"/>
     </row>
     <row r="2" spans="1:8" ht="30" customHeight="1">
-      <c r="A2" s="57" t="s">
+      <c r="A2" s="60" t="s">
         <v>86</v>
       </c>
-      <c r="B2" s="58"/>
-      <c r="C2" s="58"/>
-      <c r="D2" s="58"/>
-      <c r="E2" s="58"/>
-      <c r="F2" s="58"/>
-      <c r="G2" s="58"/>
-      <c r="H2" s="59"/>
+      <c r="B2" s="61"/>
+      <c r="C2" s="61"/>
+      <c r="D2" s="61"/>
+      <c r="E2" s="61"/>
+      <c r="F2" s="61"/>
+      <c r="G2" s="61"/>
+      <c r="H2" s="62"/>
     </row>
     <row r="3" spans="1:8" ht="25" customHeight="1">
       <c r="A3" s="2"/>
@@ -18788,32 +18830,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="38.049999999999997" customHeight="1">
-      <c r="A1" s="54" t="s">
+      <c r="A1" s="57" t="s">
         <v>191</v>
       </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
-      <c r="F1" s="55"/>
-      <c r="G1" s="55"/>
-      <c r="H1" s="55"/>
-      <c r="I1" s="55"/>
-      <c r="J1" s="56"/>
+      <c r="B1" s="58"/>
+      <c r="C1" s="58"/>
+      <c r="D1" s="58"/>
+      <c r="E1" s="58"/>
+      <c r="F1" s="58"/>
+      <c r="G1" s="58"/>
+      <c r="H1" s="58"/>
+      <c r="I1" s="58"/>
+      <c r="J1" s="59"/>
     </row>
     <row r="2" spans="1:26" ht="30" customHeight="1">
-      <c r="A2" s="57" t="s">
+      <c r="A2" s="60" t="s">
         <v>192</v>
       </c>
-      <c r="B2" s="58"/>
-      <c r="C2" s="58"/>
-      <c r="D2" s="58"/>
-      <c r="E2" s="58"/>
-      <c r="F2" s="58"/>
-      <c r="G2" s="58"/>
-      <c r="H2" s="58"/>
-      <c r="I2" s="58"/>
-      <c r="J2" s="59"/>
+      <c r="B2" s="61"/>
+      <c r="C2" s="61"/>
+      <c r="D2" s="61"/>
+      <c r="E2" s="61"/>
+      <c r="F2" s="61"/>
+      <c r="G2" s="61"/>
+      <c r="H2" s="61"/>
+      <c r="I2" s="61"/>
+      <c r="J2" s="62"/>
     </row>
     <row r="3" spans="1:26" ht="25" customHeight="1">
       <c r="A3" s="2"/>
@@ -25826,30 +25868,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="38.049999999999997" customHeight="1">
-      <c r="A1" s="54" t="s">
+      <c r="A1" s="57" t="s">
         <v>97</v>
       </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
-      <c r="F1" s="55"/>
-      <c r="G1" s="55"/>
-      <c r="H1" s="55"/>
-      <c r="I1" s="56"/>
+      <c r="B1" s="58"/>
+      <c r="C1" s="58"/>
+      <c r="D1" s="58"/>
+      <c r="E1" s="58"/>
+      <c r="F1" s="58"/>
+      <c r="G1" s="58"/>
+      <c r="H1" s="58"/>
+      <c r="I1" s="59"/>
     </row>
     <row r="2" spans="1:26" ht="30" customHeight="1">
-      <c r="A2" s="57" t="s">
+      <c r="A2" s="60" t="s">
         <v>98</v>
       </c>
-      <c r="B2" s="58"/>
-      <c r="C2" s="58"/>
-      <c r="D2" s="58"/>
-      <c r="E2" s="58"/>
-      <c r="F2" s="58"/>
-      <c r="G2" s="58"/>
-      <c r="H2" s="58"/>
-      <c r="I2" s="59"/>
+      <c r="B2" s="61"/>
+      <c r="C2" s="61"/>
+      <c r="D2" s="61"/>
+      <c r="E2" s="61"/>
+      <c r="F2" s="61"/>
+      <c r="G2" s="61"/>
+      <c r="H2" s="61"/>
+      <c r="I2" s="62"/>
     </row>
     <row r="3" spans="1:26" ht="25" customHeight="1">
       <c r="A3" s="2"/>
@@ -26052,7 +26094,7 @@
       <c r="C8" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="D8" s="64" t="s">
+      <c r="D8" s="54" t="s">
         <v>205</v>
       </c>
       <c r="E8" s="40">
@@ -26098,7 +26140,7 @@
       <c r="C9" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="D9" s="65" t="s">
+      <c r="D9" s="55" t="s">
         <v>206</v>
       </c>
       <c r="E9" s="42">
@@ -26142,7 +26184,7 @@
       <c r="C10" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="D10" s="66" t="s">
+      <c r="D10" s="56" t="s">
         <v>209</v>
       </c>
       <c r="E10" s="40">
@@ -26179,10 +26221,18 @@
       <c r="Z10" s="1"/>
     </row>
     <row r="11" spans="1:26" ht="25" customHeight="1">
-      <c r="A11" s="28"/>
-      <c r="B11" s="25"/>
-      <c r="C11" s="25"/>
-      <c r="D11" s="25"/>
+      <c r="A11" s="28">
+        <v>46278</v>
+      </c>
+      <c r="B11" s="25" t="s">
+        <v>38</v>
+      </c>
+      <c r="C11" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="D11" s="25">
+        <v>423</v>
+      </c>
       <c r="E11" s="42"/>
       <c r="F11" s="25"/>
       <c r="G11" s="25"/>
@@ -26207,9 +26257,15 @@
       <c r="Z11" s="1"/>
     </row>
     <row r="12" spans="1:26" ht="25" customHeight="1">
-      <c r="A12" s="29"/>
-      <c r="B12" s="17"/>
-      <c r="C12" s="17"/>
+      <c r="A12" s="28">
+        <v>46278</v>
+      </c>
+      <c r="B12" s="17" t="s">
+        <v>32</v>
+      </c>
+      <c r="C12" s="17" t="s">
+        <v>15</v>
+      </c>
       <c r="D12" s="17"/>
       <c r="E12" s="40"/>
       <c r="F12" s="17"/>
@@ -26235,9 +26291,15 @@
       <c r="Z12" s="1"/>
     </row>
     <row r="13" spans="1:26" ht="25" customHeight="1">
-      <c r="A13" s="28"/>
-      <c r="B13" s="25"/>
-      <c r="C13" s="25"/>
+      <c r="A13" s="28">
+        <v>46278</v>
+      </c>
+      <c r="B13" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="C13" s="25" t="s">
+        <v>15</v>
+      </c>
       <c r="D13" s="25"/>
       <c r="E13" s="42"/>
       <c r="F13" s="25"/>
@@ -32974,32 +33036,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="38.049999999999997" customHeight="1">
-      <c r="A1" s="54" t="s">
+      <c r="A1" s="57" t="s">
         <v>109</v>
       </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
-      <c r="F1" s="55"/>
-      <c r="G1" s="55"/>
-      <c r="H1" s="55"/>
-      <c r="I1" s="55"/>
-      <c r="J1" s="56"/>
+      <c r="B1" s="58"/>
+      <c r="C1" s="58"/>
+      <c r="D1" s="58"/>
+      <c r="E1" s="58"/>
+      <c r="F1" s="58"/>
+      <c r="G1" s="58"/>
+      <c r="H1" s="58"/>
+      <c r="I1" s="58"/>
+      <c r="J1" s="59"/>
     </row>
     <row r="2" spans="1:10" ht="30" customHeight="1">
-      <c r="A2" s="57" t="s">
+      <c r="A2" s="60" t="s">
         <v>110</v>
       </c>
-      <c r="B2" s="58"/>
-      <c r="C2" s="58"/>
-      <c r="D2" s="58"/>
-      <c r="E2" s="58"/>
-      <c r="F2" s="58"/>
-      <c r="G2" s="58"/>
-      <c r="H2" s="58"/>
-      <c r="I2" s="58"/>
-      <c r="J2" s="59"/>
+      <c r="B2" s="61"/>
+      <c r="C2" s="61"/>
+      <c r="D2" s="61"/>
+      <c r="E2" s="61"/>
+      <c r="F2" s="61"/>
+      <c r="G2" s="61"/>
+      <c r="H2" s="61"/>
+      <c r="I2" s="61"/>
+      <c r="J2" s="62"/>
     </row>
     <row r="3" spans="1:10" ht="25" customHeight="1">
       <c r="A3" s="2"/>
@@ -33432,30 +33494,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="38.049999999999997" customHeight="1">
-      <c r="A1" s="54" t="s">
+      <c r="A1" s="57" t="s">
         <v>176</v>
       </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
-      <c r="F1" s="55"/>
-      <c r="G1" s="55"/>
-      <c r="H1" s="55"/>
-      <c r="I1" s="56"/>
+      <c r="B1" s="58"/>
+      <c r="C1" s="58"/>
+      <c r="D1" s="58"/>
+      <c r="E1" s="58"/>
+      <c r="F1" s="58"/>
+      <c r="G1" s="58"/>
+      <c r="H1" s="58"/>
+      <c r="I1" s="59"/>
     </row>
     <row r="2" spans="1:26" ht="30" customHeight="1">
-      <c r="A2" s="57" t="s">
+      <c r="A2" s="60" t="s">
         <v>177</v>
       </c>
-      <c r="B2" s="58"/>
-      <c r="C2" s="58"/>
-      <c r="D2" s="58"/>
-      <c r="E2" s="58"/>
-      <c r="F2" s="58"/>
-      <c r="G2" s="58"/>
-      <c r="H2" s="58"/>
-      <c r="I2" s="59"/>
+      <c r="B2" s="61"/>
+      <c r="C2" s="61"/>
+      <c r="D2" s="61"/>
+      <c r="E2" s="61"/>
+      <c r="F2" s="61"/>
+      <c r="G2" s="61"/>
+      <c r="H2" s="61"/>
+      <c r="I2" s="62"/>
     </row>
     <row r="3" spans="1:26" ht="25" customHeight="1">
       <c r="A3" s="2"/>

</xml_diff>

<commit_message>
EDU-19: class_manager: latest progress
</commit_message>
<xml_diff>
--- a/assets/deen/madrasa/class_manager.xlsx
+++ b/assets/deen/madrasa/class_manager.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\SehhaDeveloper\src\l3\edu-journey\assets\deen\madrasa\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F97A1FA-5CD9-41E7-B1B9-080268B6994C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D04C380-6FE9-44DC-AB03-EC8F88B25B10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="363" uniqueCount="211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="374" uniqueCount="210">
   <si>
     <t>Madrasa Class Dashboard</t>
   </si>
@@ -662,9 +662,6 @@
     <t>`447-448</t>
   </si>
   <si>
-    <t>548</t>
-  </si>
-  <si>
     <t>Secure</t>
   </si>
   <si>
@@ -1236,13 +1233,13 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>0.6</c:v>
+                  <c:v>0.70000000000000007</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.5</c:v>
+                  <c:v>0.66666666666666663</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.95</c:v>
+                  <c:v>0.9</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1529,7 +1526,7 @@
                 <c:formatCode>0%</c:formatCode>
                 <c:ptCount val="9"/>
                 <c:pt idx="0">
-                  <c:v>0.5</c:v>
+                  <c:v>0.70000000000000007</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -2138,7 +2135,7 @@
         <v>1</v>
       </c>
       <c r="B4" s="49" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="C4" s="46"/>
       <c r="D4" s="50" t="s">
@@ -2179,7 +2176,7 @@
       </c>
       <c r="F5" s="51">
         <f>IF(COUNTIFS(ProgressTable[Student],$B$4,ProgressTable[Mastery %],"&lt;&gt;")=0,"",AVERAGEIF(ProgressTable[Student],$B$4,ProgressTable[Mastery %]))</f>
-        <v>0.5</v>
+        <v>0.70000000000000007</v>
       </c>
       <c r="G5" s="51" t="str">
         <f>IF(COUNTIFS(AssessmentTable[Student],$B$4,AssessmentTable[Percentage],"&lt;&gt;")=0,"",AVERAGEIF(AssessmentTable[Student],$B$4,AssessmentTable[Percentage]))</f>
@@ -2205,7 +2202,7 @@
       </c>
       <c r="B6" s="16" t="str">
         <f>B4</f>
-        <v>Nafisa</v>
+        <v>Mudhir</v>
       </c>
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
@@ -2226,7 +2223,7 @@
       </c>
       <c r="B7" s="16">
         <f>IFERROR(VLOOKUP(B4,Students!$B$5:$D$50,2,FALSE),"")</f>
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="C7" s="3"/>
       <c r="D7" s="63" t="s">
@@ -2347,7 +2344,7 @@
       </c>
       <c r="B13" s="5">
         <f>IF(COUNTIFS(ProgressTable[Student],A13,ProgressTable[Mastery %],"&lt;&gt;")=0,"",AVERAGEIF(ProgressTable[Student],A13,ProgressTable[Mastery %]))</f>
-        <v>0.6</v>
+        <v>0.70000000000000007</v>
       </c>
       <c r="C13" s="5">
         <f>IF(COUNTIF(AttendanceTable[Student],A13)=0,"",(COUNTIFS(AttendanceTable[Student],A13,AttendanceTable[Status],"Present")+COUNTIFS(AttendanceTable[Student],A13,AttendanceTable[Status],"Late"))/COUNTIF(AttendanceTable[Student],A13))</f>
@@ -2378,7 +2375,7 @@
       </c>
       <c r="B14" s="5">
         <f>IF(COUNTIFS(ProgressTable[Student],A14,ProgressTable[Mastery %],"&lt;&gt;")=0,"",AVERAGEIF(ProgressTable[Student],A14,ProgressTable[Mastery %]))</f>
-        <v>0.5</v>
+        <v>0.66666666666666663</v>
       </c>
       <c r="C14" s="5">
         <f>IF(COUNTIF(AttendanceTable[Student],A14)=0,"",(COUNTIFS(AttendanceTable[Student],A14,AttendanceTable[Status],"Present")+COUNTIFS(AttendanceTable[Student],A14,AttendanceTable[Status],"Late"))/COUNTIF(AttendanceTable[Student],A14))</f>
@@ -2409,7 +2406,7 @@
       </c>
       <c r="B15" s="5">
         <f>IF(COUNTIFS(ProgressTable[Student],A15,ProgressTable[Mastery %],"&lt;&gt;")=0,"",AVERAGEIF(ProgressTable[Student],A15,ProgressTable[Mastery %]))</f>
-        <v>0.95</v>
+        <v>0.9</v>
       </c>
       <c r="C15" s="5">
         <f>IF(COUNTIF(AttendanceTable[Student],A15)=0,"",(COUNTIFS(AttendanceTable[Student],A15,AttendanceTable[Status],"Present")+COUNTIFS(AttendanceTable[Student],A15,AttendanceTable[Status],"Late"))/COUNTIF(AttendanceTable[Student],A15))</f>
@@ -2511,7 +2508,7 @@
       </c>
       <c r="B20" s="5">
         <f>IF(COUNTIFS(ProgressTable[Student],$B$4,ProgressTable[Topic Area],A20,ProgressTable[Mastery %],"&lt;&gt;")=0,"",SUMIFS(ProgressTable[Mastery %],ProgressTable[Student],$B$4,ProgressTable[Topic Area],A20)/COUNTIFS(ProgressTable[Student],$B$4,ProgressTable[Topic Area],A20,ProgressTable[Mastery %],"&lt;&gt;"))</f>
-        <v>0.5</v>
+        <v>0.70000000000000007</v>
       </c>
       <c r="C20" s="3"/>
       <c r="D20" s="53" t="s">
@@ -26140,8 +26137,8 @@
       <c r="C9" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="D9" s="55" t="s">
-        <v>206</v>
+      <c r="D9" s="55">
+        <v>547</v>
       </c>
       <c r="E9" s="42">
         <v>0.7</v>
@@ -26150,10 +26147,10 @@
         <v>56</v>
       </c>
       <c r="G9" s="25" t="s">
+        <v>206</v>
+      </c>
+      <c r="H9" s="25" t="s">
         <v>207</v>
-      </c>
-      <c r="H9" s="25" t="s">
-        <v>208</v>
       </c>
       <c r="I9" s="27"/>
       <c r="J9" s="1"/>
@@ -26185,7 +26182,7 @@
         <v>15</v>
       </c>
       <c r="D10" s="56" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="E10" s="40">
         <v>0.9</v>
@@ -26197,7 +26194,7 @@
         <v>104</v>
       </c>
       <c r="H10" s="17" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="I10" s="19" t="s">
         <v>106</v>
@@ -26233,11 +26230,21 @@
       <c r="D11" s="25">
         <v>423</v>
       </c>
-      <c r="E11" s="42"/>
-      <c r="F11" s="25"/>
-      <c r="G11" s="25"/>
-      <c r="H11" s="25"/>
-      <c r="I11" s="27"/>
+      <c r="E11" s="42">
+        <v>0.8</v>
+      </c>
+      <c r="F11" s="25" t="s">
+        <v>60</v>
+      </c>
+      <c r="G11" s="25" t="s">
+        <v>206</v>
+      </c>
+      <c r="H11" s="25" t="s">
+        <v>209</v>
+      </c>
+      <c r="I11" s="27" t="s">
+        <v>106</v>
+      </c>
       <c r="J11" s="1"/>
       <c r="K11" s="1"/>
       <c r="L11" s="1"/>
@@ -26266,12 +26273,24 @@
       <c r="C12" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="D12" s="17"/>
-      <c r="E12" s="40"/>
-      <c r="F12" s="17"/>
-      <c r="G12" s="17"/>
-      <c r="H12" s="17"/>
-      <c r="I12" s="19"/>
+      <c r="D12" s="17">
+        <v>548</v>
+      </c>
+      <c r="E12" s="40">
+        <v>0.9</v>
+      </c>
+      <c r="F12" s="17" t="s">
+        <v>60</v>
+      </c>
+      <c r="G12" s="17" t="s">
+        <v>206</v>
+      </c>
+      <c r="H12" s="17" t="s">
+        <v>209</v>
+      </c>
+      <c r="I12" s="19" t="s">
+        <v>106</v>
+      </c>
       <c r="J12" s="1"/>
       <c r="K12" s="1"/>
       <c r="L12" s="1"/>
@@ -26300,12 +26319,24 @@
       <c r="C13" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="D13" s="25"/>
-      <c r="E13" s="42"/>
-      <c r="F13" s="25"/>
-      <c r="G13" s="25"/>
-      <c r="H13" s="25"/>
-      <c r="I13" s="27"/>
+      <c r="D13" s="25">
+        <v>449</v>
+      </c>
+      <c r="E13" s="42">
+        <v>1</v>
+      </c>
+      <c r="F13" s="25" t="s">
+        <v>61</v>
+      </c>
+      <c r="G13" s="25" t="s">
+        <v>104</v>
+      </c>
+      <c r="H13" s="25" t="s">
+        <v>105</v>
+      </c>
+      <c r="I13" s="27" t="s">
+        <v>106</v>
+      </c>
       <c r="J13" s="1"/>
       <c r="K13" s="1"/>
       <c r="L13" s="1"/>

</xml_diff>